<commit_message>
docs: finalize xlsx audit reports, archive unit08 track, add new conductor tracks
</commit_message>
<xml_diff>
--- a/bus-math-nextjs/public/resources/unit02-lesson05-student.xlsx
+++ b/bus-math-nextjs/public/resources/unit02-lesson05-student.xlsx
@@ -1,37 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22228"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22755" windowHeight="14535"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22755" windowHeight="14535" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Adjustments" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjustments" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="Total_Expenses">Summary!$B$3</definedName>
     <definedName name="Total_Revenue">Summary!$B$2</definedName>
     <definedName name="Net_Income">Summary!$B$4</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,20 +50,375 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -75,27 +430,27 @@
         </is>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Total Revenue</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>18500</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Total Expenses</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>9400</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Net Income</t>
@@ -103,19 +458,24 @@
       </c>
       <c r="B4">
         <f>Total_Revenue-Total_Expenses</f>
-        <v>9100</v>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Asset</t>
@@ -142,85 +502,78 @@
         </is>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Company Van</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>32000</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>4000</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>5</v>
       </c>
-      <c r="E2"/>
-    </row>
-    <row r="3" spans="1:5">
+    </row>
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Laptop Set</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>5800</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>800</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="E3"/>
-    </row>
-    <row r="4" spans="1:5">
+    </row>
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Warehouse Shelving</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>7400</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>900</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>6</v>
       </c>
-      <c r="E4"/>
-    </row>
-    <row r="5" spans="1:5">
+    </row>
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>Software License</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>2600</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3</v>
       </c>
-      <c r="E5"/>
-    </row>
-    <row r="6" spans="1:5">
+    </row>
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>Total Annual Depreciation</t>
         </is>
       </c>
-      <c r="B6"/>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6"/>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(course): support Excel for the web
</commit_message>
<xml_diff>
--- a/bus-math-nextjs/public/resources/unit02-lesson05-student.xlsx
+++ b/bus-math-nextjs/public/resources/unit02-lesson05-student.xlsx
@@ -2,42 +2,84 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22755" windowHeight="14535" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjustments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Close Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Panel" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Total_Expenses">Summary!$B$3</definedName>
-    <definedName name="Total_Revenue">Summary!$B$2</definedName>
-    <definedName name="Net_Income">Summary!$B$4</definedName>
+    <definedName name="SuppliesUsed">'Inputs'!$B$5</definedName>
+    <definedName name="InsuranceExpired">'Inputs'!$B$6</definedName>
+    <definedName name="DepreciationExpense">'Inputs'!$B$7</definedName>
+    <definedName name="WagesAccrued">'Inputs'!$B$8</definedName>
+    <definedName name="RevenueEarned">'Inputs'!$B$9</definedName>
+    <definedName name="SelectedPeriod">'Control Panel'!$B$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Inputs'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Close Model'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Control Panel'!$A$1:$B$9</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00;[Red]($#,##0.00);-"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="000070C0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2937"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,16 +87,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE8E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -413,56 +488,137 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Amount</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TechStart Month-End Adjustment Inputs</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total Revenue</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>18500</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Total Expenses</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>9400</v>
+          <t>Enter or select the period amounts. Yellow cells are inputs.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Net Income</t>
-        </is>
-      </c>
-      <c r="B4">
-        <f>Total_Revenue-Total_Expenses</f>
-        <v/>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Maximum</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Supplies used</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>5500</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Insurance expired</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Depreciation expense</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wages accrued</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Revenue earned</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -470,110 +626,578 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Asset</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Salvage</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Useful Life (Years)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Annual Depreciation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Company Van</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TechStart Month-End Close Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Adjustment Account</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Supplies Expense</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Insurance Expense</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prepaid Insurance</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Depreciation Expense</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Accumulated Depreciation</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wages Expense</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Wages Payable</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Unearned Revenue</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Service Revenue</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Adjustment totals</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Adjustment difference</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Unadjusted Debit</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Unadjusted Credit</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Adjustment Debit</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Adjustment Credit</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted Debit</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>5500</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Prepaid Insurance</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
         <v>32000</v>
       </c>
-      <c r="C2" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
+      <c r="C23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Accumulated Depreciation</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wages Payable</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Unearned Revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Owner Capital</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Service Revenue</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Supplies Expense</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Insurance Expense</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Depreciation Expense</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wages Expense</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Adjusted trial balance totals</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Adjusted trial balance difference</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Month-End Close Control Panel</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Laptop Set</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>5800</v>
-      </c>
-      <c r="C3" t="n">
-        <v>800</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4</v>
+          <t>Selected period</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Warehouse Shelving</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>7400</v>
-      </c>
-      <c r="C4" t="n">
-        <v>900</v>
-      </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
+          <t>Total adjustment debits</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Software License</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2600</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
+          <t>Total adjustment credits</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total Annual Depreciation</t>
-        </is>
-      </c>
+          <t>Adjustment difference</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Adjusted trial balance difference</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Failed validation checks</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CloseStatus</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Complete"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="notEqual" dxfId="1">
+      <formula>"Complete"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(course): support Excel for the web (#122)
* chore(measure): add Excel web compatibility track

* fix(course): support Excel for the web

* docs(review): correct issue count

* fix(unit02): address Excel web review
</commit_message>
<xml_diff>
--- a/bus-math-nextjs/public/resources/unit02-lesson05-student.xlsx
+++ b/bus-math-nextjs/public/resources/unit02-lesson05-student.xlsx
@@ -2,42 +2,84 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22755" windowHeight="14535" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjustments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Close Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Panel" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Total_Expenses">Summary!$B$3</definedName>
-    <definedName name="Total_Revenue">Summary!$B$2</definedName>
-    <definedName name="Net_Income">Summary!$B$4</definedName>
+    <definedName name="SuppliesUsed">'Inputs'!$B$5</definedName>
+    <definedName name="InsuranceExpired">'Inputs'!$B$6</definedName>
+    <definedName name="DepreciationExpense">'Inputs'!$B$7</definedName>
+    <definedName name="WagesAccrued">'Inputs'!$B$8</definedName>
+    <definedName name="RevenueEarned">'Inputs'!$B$9</definedName>
+    <definedName name="SelectedPeriod">'Control Panel'!$B$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Inputs'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Close Model'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Control Panel'!$A$1:$B$9</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00;[Red]($#,##0.00);-"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="000070C0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2937"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,16 +87,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE8E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -413,56 +488,137 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Amount</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TechStart Month-End Adjustment Inputs</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total Revenue</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>18500</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Total Expenses</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>9400</v>
+          <t>Enter or select the period amounts. Yellow cells are inputs.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Net Income</t>
-        </is>
-      </c>
-      <c r="B4">
-        <f>Total_Revenue-Total_Expenses</f>
-        <v/>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Maximum</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Supplies used</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>5500</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Insurance expired</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Depreciation expense</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wages accrued</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Revenue earned</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -470,110 +626,578 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Asset</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Salvage</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Useful Life (Years)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Annual Depreciation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Company Van</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TechStart Month-End Close Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Adjustment Account</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Supplies Expense</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Insurance Expense</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prepaid Insurance</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Depreciation Expense</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Accumulated Depreciation</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wages Expense</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Wages Payable</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Unearned Revenue</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Service Revenue</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Adjustment totals</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Adjustment difference</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Unadjusted Debit</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Unadjusted Credit</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Adjustment Debit</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Adjustment Credit</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted Debit</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>5500</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Prepaid Insurance</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
         <v>32000</v>
       </c>
-      <c r="C2" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
+      <c r="C23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Accumulated Depreciation</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wages Payable</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Unearned Revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Owner Capital</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Service Revenue</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Supplies Expense</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Insurance Expense</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Depreciation Expense</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wages Expense</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Adjusted trial balance totals</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Adjusted trial balance difference</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Month-End Close Control Panel</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Laptop Set</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>5800</v>
-      </c>
-      <c r="C3" t="n">
-        <v>800</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4</v>
+          <t>Selected period</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Warehouse Shelving</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>7400</v>
-      </c>
-      <c r="C4" t="n">
-        <v>900</v>
-      </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
+          <t>Total adjustment debits</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Software License</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2600</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
+          <t>Total adjustment credits</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total Annual Depreciation</t>
-        </is>
-      </c>
+          <t>Adjustment difference</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Adjusted trial balance difference</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Failed validation checks</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CloseStatus</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Complete"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="notEqual" dxfId="1">
+      <formula>"Complete"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>